<commit_message>
update new UI EF
</commit_message>
<xml_diff>
--- a/info/RegisterMappingDeltaPLC.xlsx
+++ b/info/RegisterMappingDeltaPLC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CongProfile\data\0.Work\2-Projects\20221201CheckWeightFullAutomationfFT\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF2213E-FA67-4C78-A837-F9BD6D5591CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6272FF20-912F-40CE-AA46-D4E9274B1B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BB171ED7-ABF6-402E-AA0F-37B73280C353}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
-  <si>
-    <t>D511</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>D510</t>
   </si>
@@ -143,9 +140,6 @@
     <t>D477</t>
   </si>
   <si>
-    <t>Delay sau khi doc can xong</t>
-  </si>
-  <si>
     <t>GlobalVariables.MyEvent.CountValue</t>
   </si>
   <si>
@@ -165,6 +159,21 @@
   </si>
   <si>
     <t>Light adon</t>
+  </si>
+  <si>
+    <t>thời gian chờ reset D506 (=0) sau khi ra khỏi bàn cân, để tắt đèn tháp (T2)</t>
+  </si>
+  <si>
+    <t>Delay sau khi doc can xong nếu OK thì chờ khoảng thời gian này mới cho chạy băng tải (T4)</t>
+  </si>
+  <si>
+    <t>thoi gian cho chạy băng tải đưa thùng vào, khi đùng sensor In thì cho băng tải chạy 1 khoảng thời gian canh thùng và giữa bàn cân thì dừng (T0)</t>
+  </si>
+  <si>
+    <t>Thời gian chờ để chốt scale stable (T1)</t>
+  </si>
+  <si>
+    <t>ms</t>
   </si>
 </sst>
 </file>
@@ -186,7 +195,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -199,8 +208,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -208,13 +223,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,49 +570,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1369B50A-174D-4ABB-9978-99C62BFE04E0}">
-  <dimension ref="A2:E36"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="36.125" customWidth="1"/>
+    <col min="3" max="3" width="68.625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>4607</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4606</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>4606</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4605</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2000</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>4605</v>
+        <v>4604</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2000</v>
+      </c>
+      <c r="E4" s="2">
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1">
-        <v>4604</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5">
-        <v>16</v>
+      <c r="B5" s="3">
+        <v>4603</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="3">
+        <v>5000</v>
+      </c>
+      <c r="E5" s="3">
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -579,10 +651,14 @@
         <v>4</v>
       </c>
       <c r="B6" s="1">
-        <v>4603</v>
-      </c>
-      <c r="E6">
-        <v>14</v>
+        <v>4602</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -590,13 +666,14 @@
         <v>5</v>
       </c>
       <c r="B7" s="1">
-        <v>4602</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7">
-        <v>12</v>
+        <v>4601</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -604,13 +681,14 @@
         <v>6</v>
       </c>
       <c r="B8" s="1">
-        <v>4601</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8">
-        <v>10</v>
+        <v>4600</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -618,13 +696,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="1">
-        <v>4600</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9">
-        <v>8</v>
+        <v>4599</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -632,13 +711,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="1">
-        <v>4599</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10">
-        <v>6</v>
+        <v>4598</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -646,13 +726,14 @@
         <v>9</v>
       </c>
       <c r="B11" s="1">
-        <v>4598</v>
-      </c>
-      <c r="C11" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11">
-        <v>4</v>
+        <v>4597</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -660,179 +741,204 @@
         <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>4597</v>
-      </c>
-      <c r="C12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
+        <v>4596</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1">
-        <v>4596</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
+      <c r="B13" s="2">
+        <v>4595</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14">
-        <v>4595</v>
-      </c>
+      <c r="B14" s="2">
+        <v>4594</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
-        <v>4594</v>
-      </c>
+      <c r="B15" s="2">
+        <v>4593</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16">
-        <v>4593</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B16" s="2">
+        <v>4592</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B17">
-        <v>4592</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="B17" s="2">
+        <v>4591</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B18">
-        <v>4591</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B18" s="2">
+        <v>4590</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B19">
-        <v>4590</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="B19" s="2">
+        <v>4589</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B20">
-        <v>4589</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B20" s="2">
+        <v>4588</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B21">
-        <v>4588</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B21" s="2">
+        <v>4587</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B22">
-        <v>4587</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B22" s="2">
+        <v>4586</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>21</v>
       </c>
       <c r="B23">
-        <v>4586</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4585</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>22</v>
       </c>
       <c r="B24">
-        <v>4585</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4584</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>23</v>
       </c>
       <c r="B25">
-        <v>4584</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4583</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>4583</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4582</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>25</v>
       </c>
       <c r="B27">
-        <v>4582</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4581</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>26</v>
       </c>
       <c r="B28">
-        <v>4581</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4580</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>27</v>
       </c>
       <c r="B29">
-        <v>4580</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4579</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>28</v>
       </c>
       <c r="B30">
-        <v>4579</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4578</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>29</v>
       </c>
       <c r="B31">
-        <v>4578</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4577</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>30</v>
       </c>
       <c r="B32">
-        <v>4577</v>
+        <v>4576</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -840,7 +946,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>4576</v>
+        <v>4575</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -848,7 +954,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>4575</v>
+        <v>4574</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
@@ -856,14 +962,6 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>4574</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>34</v>
-      </c>
-      <c r="B36">
         <v>4573</v>
       </c>
     </row>

</xml_diff>